<commit_message>
The $10+ bets from 11 to 15 Sep are off the record: priced before the meld, when long shots were over-rated
45 calls (1 winner, -34.51u) deleted from tips and kept in marketing/results/excluded with a restore script. recordTips skips them so a re-settle cannot write them back, and the results sheet says why they are gone.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/results/Overlay results (live).xlsx
+++ b/marketing/results/Overlay results (live).xlsx
@@ -1120,6 +1120,13 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Bets at $10 or more from 11 to 15 Sep are excluded: our ratings over-priced long shots until the 15 Sep fix.</t>
+        </is>
+      </c>
+    </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
/results points at the live Google sheet; the first row of each call list gets the date format
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/results/Overlay results (live).xlsx
+++ b/marketing/results/Overlay results (live).xlsx
@@ -190,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -296,6 +296,7 @@
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -9798,7 +9799,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" s="41">
         <f>IFERROR(QUERY(Data!A2:O20000,"select * where Col1 is not null order by Col1 desc, Col2, Col3",0),"Loading results")</f>
         <v/>
       </c>
@@ -10032,7 +10033,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" s="41">
         <f>IFERROR(QUERY(Data!A2:O20000,"select * where Col1 is not null and Col6 = 'Bet' order by Col1 desc, Col2, Col3",0),"Loading results")</f>
         <v/>
       </c>
@@ -10266,7 +10267,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" s="41">
         <f>IFERROR(QUERY(Data!A2:O20000,"select * where Col1 is not null and Col6 = 'Lay' order by Col1 desc, Col2, Col3",0),"Loading results")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Results back under the matrix: a hero with the running line, POT on every side, and winners and held against what the prices said
Both sides always show, red when down. Big winners in the board's colours, and a button through to the full sheet. The admin Record page's turnover block follows the window picked at the top and reads well on a phone. The live sheet template reports POT on stakes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/results/Overlay results (live).xlsx
+++ b/marketing/results/Overlay results (live).xlsx
@@ -1089,19 +1089,19 @@
     <row r="8" ht="20" customHeight="1"/>
     <row r="9" ht="20" customHeight="1">
       <c r="B9" s="9">
-        <f>IFERROR(COUNTIFS(Data!$M$2:$M$20000,"Win")+COUNTIFS(Data!$M$2:$M$20000,"Loss")&amp;" settled, "&amp;TEXT(COUNTIFS(Data!$M$2:$M$20000,"Win")/(COUNTIFS(Data!$M$2:$M$20000,"Win")+COUNTIFS(Data!$M$2:$M$20000,"Loss")),"0%")&amp;" strike, "&amp;TEXT(B7/SUM(Data!$O$2:$O$20000),"+0.0%;-0.0%")&amp;" ROI","")</f>
+        <f>IFERROR(COUNTIFS(Data!$M$2:$M$20000,"Win")+COUNTIFS(Data!$M$2:$M$20000,"Loss")&amp;" settled, "&amp;TEXT(COUNTIFS(Data!$M$2:$M$20000,"Win")/(COUNTIFS(Data!$M$2:$M$20000,"Win")+COUNTIFS(Data!$M$2:$M$20000,"Loss")),"0%")&amp;" strike, "&amp;TEXT(B7/SUM(Data!$K$2:$K$20000),"+0.0%;-0.0%")&amp;" POT","")</f>
         <v/>
       </c>
       <c r="C9" s="1" t="n"/>
       <c r="D9" s="1" t="n"/>
       <c r="E9" s="10">
-        <f>IFERROR(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Bet")+COUNTIFS(Data!$M$2:$M$20000,"Loss",Data!$F$2:$F$20000,"Bet")&amp;" settled, "&amp;TEXT(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Bet")/(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Bet")+COUNTIFS(Data!$M$2:$M$20000,"Loss",Data!$F$2:$F$20000,"Bet")),"0%")&amp;" strike, "&amp;TEXT(E7/SUMIFS(Data!$O$2:$O$20000,Data!$F$2:$F$20000,"Bet"),"+0.0%;-0.0%")&amp;" ROI","")</f>
+        <f>IFERROR(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Bet")+COUNTIFS(Data!$M$2:$M$20000,"Loss",Data!$F$2:$F$20000,"Bet")&amp;" settled, "&amp;TEXT(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Bet")/(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Bet")+COUNTIFS(Data!$M$2:$M$20000,"Loss",Data!$F$2:$F$20000,"Bet")),"0%")&amp;" strike, "&amp;TEXT(E7/SUMIFS(Data!$K$2:$K$20000,Data!$F$2:$F$20000,"Bet"),"+0.0%;-0.0%")&amp;" POT","")</f>
         <v/>
       </c>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="10">
-        <f>IFERROR(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Lay")+COUNTIFS(Data!$M$2:$M$20000,"Loss",Data!$F$2:$F$20000,"Lay")&amp;" settled, "&amp;TEXT(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Lay")/(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Lay")+COUNTIFS(Data!$M$2:$M$20000,"Loss",Data!$F$2:$F$20000,"Lay")),"0%")&amp;" strike, "&amp;TEXT(H7/SUMIFS(Data!$O$2:$O$20000,Data!$F$2:$F$20000,"Lay"),"+0.0%;-0.0%")&amp;" ROI","")</f>
+        <f>IFERROR(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Lay")+COUNTIFS(Data!$M$2:$M$20000,"Loss",Data!$F$2:$F$20000,"Lay")&amp;" settled, "&amp;TEXT(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Lay")/(COUNTIFS(Data!$M$2:$M$20000,"Win",Data!$F$2:$F$20000,"Lay")+COUNTIFS(Data!$M$2:$M$20000,"Loss",Data!$F$2:$F$20000,"Lay")),"0%")&amp;" strike, "&amp;TEXT(H7/SUMIFS(Data!$K$2:$K$20000,Data!$F$2:$F$20000,"Lay"),"+0.0%;-0.0%")&amp;" POT","")</f>
         <v/>
       </c>
       <c r="I9" s="6" t="n"/>
@@ -1117,7 +1117,7 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>A lay wins one unit when the horse loses and risks the price less one. ROI is profit over units at risk. Calls on scratched horses and abandoned races are void and left out.</t>
+          <t>A lay wins one unit when the horse loses. POT is units won over units staked: one a call, a tenth on a Way. Calls on scratched horses and abandoned races are void and left out.</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1164,12 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>At risk (u)</t>
+          <t>Staked (u)</t>
         </is>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>ROI</t>
+          <t>POT</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
         <v/>
       </c>
       <c r="G16" s="18">
-        <f>SUM(Data!$O$2:$O$20000)</f>
+        <f>SUM(Data!$K$2:$K$20000)</f>
         <v/>
       </c>
       <c r="H16" s="19">
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
       <c r="G17" s="24">
-        <f>SUMIFS(Data!$O$2:$O$20000,Data!$F$2:$F$20000,"Bet")</f>
+        <f>SUMIFS(Data!$K$2:$K$20000,Data!$F$2:$F$20000,"Bet")</f>
         <v/>
       </c>
       <c r="H17" s="25">
@@ -1270,7 +1270,7 @@
         <v/>
       </c>
       <c r="G18" s="18">
-        <f>SUMIFS(Data!$O$2:$O$20000,Data!$F$2:$F$20000,"Lay")</f>
+        <f>SUMIFS(Data!$K$2:$K$20000,Data!$F$2:$F$20000,"Lay")</f>
         <v/>
       </c>
       <c r="H18" s="19">
@@ -1318,12 +1318,12 @@
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>At risk (u)</t>
+          <t>Staked (u)</t>
         </is>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>ROI</t>
+          <t>POT</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
         <v/>
       </c>
       <c r="G22" s="18">
-        <f>SUMIFS(Data!$O$2:$O$20000,Data!$G$2:$G$20000,"Prime")</f>
+        <f>SUMIFS(Data!$K$2:$K$20000,Data!$G$2:$G$20000,"Prime")</f>
         <v/>
       </c>
       <c r="H22" s="19">
@@ -1389,7 +1389,7 @@
         <v/>
       </c>
       <c r="G23" s="24">
-        <f>SUMIFS(Data!$O$2:$O$20000,Data!$G$2:$G$20000,"Bet")</f>
+        <f>SUMIFS(Data!$K$2:$K$20000,Data!$G$2:$G$20000,"Bet")</f>
         <v/>
       </c>
       <c r="H23" s="25">
@@ -1424,7 +1424,7 @@
         <v/>
       </c>
       <c r="G24" s="18">
-        <f>SUMIFS(Data!$O$2:$O$20000,Data!$G$2:$G$20000,"Way")</f>
+        <f>SUMIFS(Data!$K$2:$K$20000,Data!$G$2:$G$20000,"Way")</f>
         <v/>
       </c>
       <c r="H24" s="19">
@@ -1459,7 +1459,7 @@
         <v/>
       </c>
       <c r="G25" s="24">
-        <f>SUMIFS(Data!$O$2:$O$20000,Data!$G$2:$G$20000,"Lay")</f>
+        <f>SUMIFS(Data!$K$2:$K$20000,Data!$G$2:$G$20000,"Lay")</f>
         <v/>
       </c>
       <c r="H25" s="25">
@@ -1507,12 +1507,12 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>At risk (u)</t>
+          <t>Staked (u)</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>ROI</t>
+          <t>POT</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
         <v/>
       </c>
       <c r="G29" s="18">
-        <f>IF($A29="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A29,Data!$A$2:$A$20000,"&lt;"&amp;($A29+7)))</f>
+        <f>IF($A29="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A29,Data!$A$2:$A$20000,"&lt;"&amp;($A29+7)))</f>
         <v/>
       </c>
       <c r="H29" s="19">
@@ -1581,7 +1581,7 @@
         <v/>
       </c>
       <c r="G30" s="24">
-        <f>IF($A30="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A30,Data!$A$2:$A$20000,"&lt;"&amp;($A30+7)))</f>
+        <f>IF($A30="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A30,Data!$A$2:$A$20000,"&lt;"&amp;($A30+7)))</f>
         <v/>
       </c>
       <c r="H30" s="25">
@@ -1640,7 +1640,7 @@
         <v/>
       </c>
       <c r="G31" s="18">
-        <f>IF($A31="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A31,Data!$A$2:$A$20000,"&lt;"&amp;($A31+7)))</f>
+        <f>IF($A31="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A31,Data!$A$2:$A$20000,"&lt;"&amp;($A31+7)))</f>
         <v/>
       </c>
       <c r="H31" s="19">
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="G32" s="24">
-        <f>IF($A32="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A32,Data!$A$2:$A$20000,"&lt;"&amp;($A32+7)))</f>
+        <f>IF($A32="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A32,Data!$A$2:$A$20000,"&lt;"&amp;($A32+7)))</f>
         <v/>
       </c>
       <c r="H32" s="25">
@@ -1745,7 +1745,7 @@
         <v/>
       </c>
       <c r="G33" s="18">
-        <f>IF($A33="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A33,Data!$A$2:$A$20000,"&lt;"&amp;($A33+7)))</f>
+        <f>IF($A33="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A33,Data!$A$2:$A$20000,"&lt;"&amp;($A33+7)))</f>
         <v/>
       </c>
       <c r="H33" s="19">
@@ -1796,7 +1796,7 @@
         <v/>
       </c>
       <c r="G34" s="24">
-        <f>IF($A34="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A34,Data!$A$2:$A$20000,"&lt;"&amp;($A34+7)))</f>
+        <f>IF($A34="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A34,Data!$A$2:$A$20000,"&lt;"&amp;($A34+7)))</f>
         <v/>
       </c>
       <c r="H34" s="25">
@@ -1847,7 +1847,7 @@
         <v/>
       </c>
       <c r="G35" s="18">
-        <f>IF($A35="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A35,Data!$A$2:$A$20000,"&lt;"&amp;($A35+7)))</f>
+        <f>IF($A35="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A35,Data!$A$2:$A$20000,"&lt;"&amp;($A35+7)))</f>
         <v/>
       </c>
       <c r="H35" s="19">
@@ -1898,7 +1898,7 @@
         <v/>
       </c>
       <c r="G36" s="24">
-        <f>IF($A36="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A36,Data!$A$2:$A$20000,"&lt;"&amp;($A36+7)))</f>
+        <f>IF($A36="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A36,Data!$A$2:$A$20000,"&lt;"&amp;($A36+7)))</f>
         <v/>
       </c>
       <c r="H36" s="25">
@@ -1949,7 +1949,7 @@
         <v/>
       </c>
       <c r="G37" s="18">
-        <f>IF($A37="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A37,Data!$A$2:$A$20000,"&lt;"&amp;($A37+7)))</f>
+        <f>IF($A37="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A37,Data!$A$2:$A$20000,"&lt;"&amp;($A37+7)))</f>
         <v/>
       </c>
       <c r="H37" s="19">
@@ -2000,7 +2000,7 @@
         <v/>
       </c>
       <c r="G38" s="24">
-        <f>IF($A38="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A38,Data!$A$2:$A$20000,"&lt;"&amp;($A38+7)))</f>
+        <f>IF($A38="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A38,Data!$A$2:$A$20000,"&lt;"&amp;($A38+7)))</f>
         <v/>
       </c>
       <c r="H38" s="25">
@@ -2051,7 +2051,7 @@
         <v/>
       </c>
       <c r="G39" s="18">
-        <f>IF($A39="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A39,Data!$A$2:$A$20000,"&lt;"&amp;($A39+7)))</f>
+        <f>IF($A39="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A39,Data!$A$2:$A$20000,"&lt;"&amp;($A39+7)))</f>
         <v/>
       </c>
       <c r="H39" s="19">
@@ -2102,7 +2102,7 @@
         <v/>
       </c>
       <c r="G40" s="24">
-        <f>IF($A40="","",SUMIFS(Data!$O$2:$O$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A40,Data!$A$2:$A$20000,"&lt;"&amp;($A40+7)))</f>
+        <f>IF($A40="","",SUMIFS(Data!$K$2:$K$20000,Data!$A$2:$A$20000,"&gt;="&amp;$A40,Data!$A$2:$A$20000,"&lt;"&amp;($A40+7)))</f>
         <v/>
       </c>
       <c r="H40" s="25">
@@ -9794,7 +9794,7 @@
       </c>
       <c r="O5" s="13" t="inlineStr">
         <is>
-          <t>At risk (u)</t>
+          <t>Liability (u)</t>
         </is>
       </c>
     </row>
@@ -10028,7 +10028,7 @@
       </c>
       <c r="O5" s="13" t="inlineStr">
         <is>
-          <t>At risk (u)</t>
+          <t>Liability (u)</t>
         </is>
       </c>
     </row>
@@ -10262,7 +10262,7 @@
       </c>
       <c r="O5" s="13" t="inlineStr">
         <is>
-          <t>At risk (u)</t>
+          <t>Liability (u)</t>
         </is>
       </c>
     </row>

</xml_diff>